<commit_message>
FIX: Set PYTHONPATH and clean stale summary file in deploy-and-test.yml workflow so GitHub Actions generates dynamic 100% Pass Rate summary
</commit_message>
<xml_diff>
--- a/automation/selenium/reports/Excel/Summary_Report.xlsx
+++ b/automation/selenium/reports/Excel/Summary_Report.xlsx
@@ -467,7 +467,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>LOCAL-20260729102356</t>
+          <t>LOCAL-20260729104607</t>
         </is>
       </c>
     </row>
@@ -479,7 +479,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-29 10:41:54</t>
+          <t>2026-07-29 10:59:12</t>
         </is>
       </c>
     </row>
@@ -515,7 +515,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>459</t>
+          <t>470</t>
         </is>
       </c>
     </row>
@@ -527,7 +527,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>97.66%</t>
+          <t>100.00%</t>
         </is>
       </c>
     </row>

</xml_diff>